<commit_message>
feat: add Security Summary tab to Vulnerability Analysis Report
</commit_message>
<xml_diff>
--- a/tests/reports/Vulnerability_Analysis_Report.xlsx
+++ b/tests/reports/Vulnerability_Analysis_Report.xlsx
@@ -5,18 +5,19 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Security Analysis" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Security Summary" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="63">
   <si>
     <t>PAYBUDDY SECURITY &amp; VULNERABILITY ANALYSIS REPORT</t>
   </si>
   <si>
-    <t>Generated: 16/6/2026, 2:13:20 pm | Scans Completed: 10 | Status: SECURE</t>
+    <t>Generated: 16/6/2026, 2:33:53 pm | Scans Completed: 10 | Status: SECURE</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -155,13 +156,58 @@
   </si>
   <si>
     <t>User session details stored locally in browser session.</t>
+  </si>
+  <si>
+    <t>PAYBUDDY WEB SECURITY REPORT</t>
+  </si>
+  <si>
+    <t>Scan Date</t>
+  </si>
+  <si>
+    <t>16-Jun-2026</t>
+  </si>
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>Total Test Cases</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Skipped</t>
+  </si>
+  <si>
+    <t>Pass Percentage</t>
+  </si>
+  <si>
+    <t>100%</t>
+  </si>
+  <si>
+    <t>Severity Level</t>
+  </si>
+  <si>
+    <t>Moderate</t>
+  </si>
+  <si>
+    <t>Informational</t>
+  </si>
+  <si>
+    <t>OVERALL STATUS</t>
+  </si>
+  <si>
+    <t>PASS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -209,8 +255,31 @@
       <sz val="10"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="14"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF065F46"/>
+      <sz val="11"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -237,8 +306,13 @@
         <fgColor rgb="D1FAE5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF374151"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -268,11 +342,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFE5E7EB"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF111827"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -296,6 +381,27 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -891,4 +997,141 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="3" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: optimize vulnerability report styling and summary metrics
</commit_message>
<xml_diff>
--- a/tests/reports/Vulnerability_Analysis_Report.xlsx
+++ b/tests/reports/Vulnerability_Analysis_Report.xlsx
@@ -12,12 +12,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="62">
   <si>
     <t>PAYBUDDY SECURITY &amp; VULNERABILITY ANALYSIS REPORT</t>
   </si>
   <si>
-    <t>Generated: 16/6/2026, 2:33:53 pm | Scans Completed: 10 | Status: SECURE</t>
+    <t>Generated: 16/6/2026, 2:45:13 pm | Scans Completed: 10 | Status: SECURE</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -47,154 +47,151 @@
     <t>Check third-party package vulnerabilities</t>
   </si>
   <si>
+    <t>Informational</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>Zero security vulnerabilities detected in production packages.</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-001</t>
+  </si>
+  <si>
+    <t>Access Control</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated read rejection</t>
+  </si>
+  <si>
+    <t>Database correctly rejected unauthorized read request (403 Forbidden).</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-002</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated write rejection</t>
+  </si>
+  <si>
+    <t>Database correctly rejected unauthorized write attempt.</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-001</t>
+  </si>
+  <si>
+    <t>Data Security</t>
+  </si>
+  <si>
+    <t>SSL Certificate Verification</t>
+  </si>
+  <si>
+    <t>Production deployment strictly uses encrypted HTTPS connection.</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-001</t>
+  </si>
+  <si>
+    <t>Input Validation</t>
+  </si>
+  <si>
+    <t>Password masking verification</t>
+  </si>
+  <si>
+    <t>Sensitive credentials masked with password type configuration.</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-002</t>
+  </si>
+  <si>
+    <t>Mandatory input validation constraints</t>
+  </si>
+  <si>
+    <t>Email validation constraint is active on login form.</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-003</t>
+  </si>
+  <si>
+    <t>Secure dashboard route protection</t>
+  </si>
+  <si>
+    <t>Route security validated. Successful login redirects to authorized view.</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-001</t>
+  </si>
+  <si>
+    <t>XSS Prevention</t>
+  </si>
+  <si>
+    <t>XSS escaping on Customer creation</t>
+  </si>
+  <si>
+    <t>XSS payload successfully escaped and rendered as safe plain text.</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-002</t>
+  </si>
+  <si>
+    <t>XSS escaping on Sales creation</t>
+  </si>
+  <si>
+    <t>HTML image payload successfully escaped and displayed safely.</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-002</t>
+  </si>
+  <si>
+    <t>Secure sessions state validation</t>
+  </si>
+  <si>
+    <t>User session details stored locally in browser session.</t>
+  </si>
+  <si>
+    <t>PAYBUDDY WEB SECURITY REPORT</t>
+  </si>
+  <si>
+    <t>Scan Date</t>
+  </si>
+  <si>
+    <t>16-Jun-2026</t>
+  </si>
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>Total Test Cases</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Skipped</t>
+  </si>
+  <si>
+    <t>Pass Percentage</t>
+  </si>
+  <si>
+    <t>100%</t>
+  </si>
+  <si>
+    <t>Severity Level</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
     <t>High</t>
   </si>
   <si>
-    <t>Passed</t>
-  </si>
-  <si>
-    <t>Zero security vulnerabilities detected in production packages.</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-001</t>
-  </si>
-  <si>
-    <t>Access Control</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated read rejection</t>
-  </si>
-  <si>
-    <t>Database correctly rejected unauthorized read request (403 Forbidden).</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-002</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated write rejection</t>
-  </si>
-  <si>
-    <t>Critical</t>
-  </si>
-  <si>
-    <t>Database correctly rejected unauthorized write attempt.</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-001</t>
-  </si>
-  <si>
-    <t>Data Security</t>
-  </si>
-  <si>
-    <t>SSL Certificate Verification</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>Production deployment strictly uses encrypted HTTPS connection.</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-001</t>
-  </si>
-  <si>
-    <t>Input Validation</t>
-  </si>
-  <si>
-    <t>Password masking verification</t>
-  </si>
-  <si>
-    <t>Sensitive credentials masked with password type configuration.</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-002</t>
-  </si>
-  <si>
-    <t>Mandatory input validation constraints</t>
+    <t>Moderate</t>
   </si>
   <si>
     <t>Low</t>
-  </si>
-  <si>
-    <t>Email validation constraint is active on login form.</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-003</t>
-  </si>
-  <si>
-    <t>Secure dashboard route protection</t>
-  </si>
-  <si>
-    <t>Route security validated. Successful login redirects to authorized view.</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-001</t>
-  </si>
-  <si>
-    <t>XSS Prevention</t>
-  </si>
-  <si>
-    <t>XSS escaping on Customer creation</t>
-  </si>
-  <si>
-    <t>XSS payload successfully escaped and rendered as safe plain text.</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-002</t>
-  </si>
-  <si>
-    <t>XSS escaping on Sales creation</t>
-  </si>
-  <si>
-    <t>HTML image payload successfully escaped and displayed safely.</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-002</t>
-  </si>
-  <si>
-    <t>Secure sessions state validation</t>
-  </si>
-  <si>
-    <t>User session details stored locally in browser session.</t>
-  </si>
-  <si>
-    <t>PAYBUDDY WEB SECURITY REPORT</t>
-  </si>
-  <si>
-    <t>Scan Date</t>
-  </si>
-  <si>
-    <t>16-Jun-2026</t>
-  </si>
-  <si>
-    <t>Metric</t>
-  </si>
-  <si>
-    <t>Count</t>
-  </si>
-  <si>
-    <t>Total Test Cases</t>
-  </si>
-  <si>
-    <t>Failed</t>
-  </si>
-  <si>
-    <t>Skipped</t>
-  </si>
-  <si>
-    <t>Pass Percentage</t>
-  </si>
-  <si>
-    <t>100%</t>
-  </si>
-  <si>
-    <t>Severity Level</t>
-  </si>
-  <si>
-    <t>Moderate</t>
-  </si>
-  <si>
-    <t>Informational</t>
   </si>
   <si>
     <t>OVERALL STATUS</t>
@@ -207,7 +204,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -239,19 +236,7 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF990000"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
       <color rgb="FF065F46"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFB36600"/>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
@@ -357,7 +342,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -371,37 +356,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -840,84 +819,84 @@
         <v>19</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>12</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>25</v>
+      <c r="D8" s="5" t="s">
+        <v>11</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>12</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>25</v>
+      <c r="D9" s="5" t="s">
+        <v>11</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>12</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>33</v>
+        <v>30</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>11</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>12</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>11</v>
@@ -926,18 +905,18 @@
         <v>12</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>11</v>
@@ -946,18 +925,18 @@
         <v>12</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>11</v>
@@ -966,27 +945,27 @@
         <v>12</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>33</v>
+        <v>43</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>11</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>12</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1009,38 +988,38 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+      <c r="B5" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="11" t="s">
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="B6" s="8">
+      <c r="B6" s="5">
         <v>10</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="11" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="6">
@@ -1048,83 +1027,83 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B8" s="8">
+    </row>
+    <row r="12" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="B9" s="8">
+    <row r="14" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B14" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
+    <row r="15" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="B12" s="12" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
+      <c r="B15" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="B15" s="8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="B16" s="8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
+      <c r="B17" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" ht="25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
+      <c r="B19" s="13" t="s">
         <v>61</v>
-      </c>
-      <c r="B19" s="15" t="s">
-        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: clean vulnerability report and add more checks
</commit_message>
<xml_diff>
--- a/tests/reports/Vulnerability_Analysis_Report.xlsx
+++ b/tests/reports/Vulnerability_Analysis_Report.xlsx
@@ -12,12 +12,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="86">
   <si>
     <t>PAYBUDDY SECURITY &amp; VULNERABILITY ANALYSIS REPORT</t>
   </si>
   <si>
-    <t>Generated: 16/6/2026, 2:45:13 pm | Scans Completed: 10 | Status: SECURE</t>
+    <t>Generated: 16/6/2026, 2:59:41 pm | Scans Completed: 31 | Status: SECURE</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -29,15 +29,9 @@
     <t>Vulnerability Checked</t>
   </si>
   <si>
-    <t>Risk Level</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
-    <t>Remarks</t>
-  </si>
-  <si>
     <t>TC-SEC-DEP-001</t>
   </si>
   <si>
@@ -47,48 +41,93 @@
     <t>Check third-party package vulnerabilities</t>
   </si>
   <si>
-    <t>Informational</t>
-  </si>
-  <si>
     <t>Passed</t>
   </si>
   <si>
-    <t>Zero security vulnerabilities detected in production packages.</t>
-  </si>
-  <si>
     <t>TC-SEC-AUTH-001</t>
   </si>
   <si>
     <t>Access Control</t>
   </si>
   <si>
-    <t>Verify unauthenticated read rejection</t>
-  </si>
-  <si>
-    <t>Database correctly rejected unauthorized read request (403 Forbidden).</t>
+    <t>Verify unauthenticated read rejection (customers)</t>
   </si>
   <si>
     <t>TC-SEC-AUTH-002</t>
   </si>
   <si>
-    <t>Verify unauthenticated write rejection</t>
-  </si>
-  <si>
-    <t>Database correctly rejected unauthorized write attempt.</t>
+    <t>Verify unauthenticated write rejection (customers)</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-003</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated read rejection (sales)</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-004</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated write rejection (sales)</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-005</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated write rejection (payments)</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-006</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated write rejection (installments)</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-007</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated write rejection (ledger)</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-015</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated read rejection (payments)</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-016</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated read rejection (installments)</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-017</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated read rejection (ledger)</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-003</t>
+  </si>
+  <si>
+    <t>Data Security</t>
+  </si>
+  <si>
+    <t>Verify X-Content-Type-Options: nosniff header present</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-004</t>
+  </si>
+  <si>
+    <t>Verify Clickjacking protection (X-Frame-Options/CSP)</t>
   </si>
   <si>
     <t>TC-SEC-CONF-001</t>
   </si>
   <si>
-    <t>Data Security</t>
-  </si>
-  <si>
     <t>SSL Certificate Verification</t>
   </si>
   <si>
-    <t>Production deployment strictly uses encrypted HTTPS connection.</t>
-  </si>
-  <si>
     <t>TC-SEC-VAL-001</t>
   </si>
   <si>
@@ -98,37 +137,73 @@
     <t>Password masking verification</t>
   </si>
   <si>
-    <t>Sensitive credentials masked with password type configuration.</t>
-  </si>
-  <si>
     <t>TC-SEC-VAL-002</t>
   </si>
   <si>
     <t>Mandatory input validation constraints</t>
   </si>
   <si>
-    <t>Email validation constraint is active on login form.</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-003</t>
-  </si>
-  <si>
-    <t>Secure dashboard route protection</t>
-  </si>
-  <si>
-    <t>Route security validated. Successful login redirects to authorized view.</t>
+    <t>TC-SEC-AUTH-008</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated dashboard access block</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-009</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated customers access block</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-010</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated sales access block</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-011</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated payments access block</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-012</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated installments access block</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-013</t>
+  </si>
+  <si>
+    <t>Verify unauthenticated ledger access block</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-014</t>
+  </si>
+  <si>
+    <t>Verify post-login authenticated redirect</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-005</t>
+  </si>
+  <si>
+    <t>Verify raw password is not stored in localStorage</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-004</t>
+  </si>
+  <si>
+    <t>XSS Prevention</t>
+  </si>
+  <si>
+    <t>Verify XSS input validation constraint on phone number</t>
   </si>
   <si>
     <t>TC-SEC-XSS-001</t>
   </si>
   <si>
-    <t>XSS Prevention</t>
-  </si>
-  <si>
-    <t>XSS escaping on Customer creation</t>
-  </si>
-  <si>
-    <t>XSS payload successfully escaped and rendered as safe plain text.</t>
+    <t>XSS escaping on Customer creation name field</t>
   </si>
   <si>
     <t>TC-SEC-XSS-002</t>
@@ -137,7 +212,16 @@
     <t>XSS escaping on Sales creation</t>
   </si>
   <si>
-    <t>HTML image payload successfully escaped and displayed safely.</t>
+    <t>TC-SEC-VAL-003</t>
+  </si>
+  <si>
+    <t>SQL Injection boundary input escaping check</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-005</t>
+  </si>
+  <si>
+    <t>HTML escaping check on Payments input</t>
   </si>
   <si>
     <t>TC-SEC-CONF-002</t>
@@ -146,7 +230,10 @@
     <t>Secure sessions state validation</t>
   </si>
   <si>
-    <t>User session details stored locally in browser session.</t>
+    <t>TC-SEC-AUTH-018</t>
+  </si>
+  <si>
+    <t>Verify session termination and login redirect on logout</t>
   </si>
   <si>
     <t>PAYBUDDY WEB SECURITY REPORT</t>
@@ -177,21 +264,6 @@
   </si>
   <si>
     <t>100%</t>
-  </si>
-  <si>
-    <t>Severity Level</t>
-  </si>
-  <si>
-    <t>Critical</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>Moderate</t>
-  </si>
-  <si>
-    <t>Low</t>
   </si>
   <si>
     <t>OVERALL STATUS</t>
@@ -356,9 +428,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -376,6 +445,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -722,33 +794,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="6" width="60" customWidth="1"/>
+    <col min="1" max="4" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" ht="40" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="4" ht="25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" ht="25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -761,217 +829,445 @@
       <c r="D4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="6" t="s">
+      <c r="B6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="D6" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="B7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="D7" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="B8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="4" t="s">
+      <c r="D8" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="B9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="D9" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="4" t="s">
+      <c r="B10" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="D10" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B11" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D11" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="4" t="s">
+      <c r="B12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="D12" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B13" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D13" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="4" t="s">
+      <c r="B14" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="10" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="D14" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="4" t="s">
+      <c r="B15" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="4" t="s">
+      <c r="D15" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="11" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="B16" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="4" t="s">
+      <c r="C16" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="4" t="s">
+      <c r="D16" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="12" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="B17" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="D17" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="B18" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="4" t="s">
+      <c r="D18" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="13" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+      <c r="B19" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C13" s="4" t="s">
+      <c r="C19" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="4" t="s">
+      <c r="D19" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="14" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+      <c r="B20" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="4" t="s">
+      <c r="D20" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" s="4" t="s">
+      <c r="B21" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>44</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -980,7 +1276,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -988,122 +1284,74 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
+      <c r="A1" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>47</v>
+      <c r="A3" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>49</v>
+      <c r="A5" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" s="5">
-        <v>10</v>
+      <c r="A6" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="11">
+        <v>31</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="6">
-        <v>10</v>
+      <c r="A7" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="5">
+        <v>31</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="B8" s="5">
+      <c r="A8" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B8" s="11">
         <v>0</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="B9" s="5">
+      <c r="A9" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" s="11">
         <v>0</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="B13" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="B14" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="B15" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B16" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B17" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" ht="25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>61</v>
+      <c r="A10" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="12" ht="25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ci: expand security scanning suite to run exactly 124 vulnerability test cases
</commit_message>
<xml_diff>
--- a/tests/reports/Vulnerability_Analysis_Report.xlsx
+++ b/tests/reports/Vulnerability_Analysis_Report.xlsx
@@ -12,12 +12,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="272">
   <si>
     <t>PAYBUDDY SECURITY &amp; VULNERABILITY ANALYSIS REPORT</t>
   </si>
   <si>
-    <t>Generated: 16/6/2026, 2:59:41 pm | Scans Completed: 31 | Status: SECURE</t>
+    <t>Generated: 22/6/2026, 9:35:04 am | Scans Completed: 124 | Status: SECURE</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -32,6 +32,447 @@
     <t>Status</t>
   </si>
   <si>
+    <t>TC-SEC-AUTH-014</t>
+  </si>
+  <si>
+    <t>Access Control</t>
+  </si>
+  <si>
+    <t>Verify post-login authenticated redirect</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-018</t>
+  </si>
+  <si>
+    <t>Verify session termination and login redirect on logout</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-AUDI</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'audit_trail' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-CUST</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'customers' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-DATA</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'database_backups' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-INST</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'installments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-LEDG</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'ledger' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-PAYM</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'payments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-SALE</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'sales' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-SETT</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'settings' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-SYST</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'system_logs' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-USER</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'users' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-AUDI</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'audit_trail' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-CUST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'customers' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-DATA</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'database_backups' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-INST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'installments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-LEDG</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'ledger' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-PAYM</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'payments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-SALE</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'sales' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-SETT</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'settings' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-SYST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'system_logs' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-USER</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'users' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-AUDI</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'audit_trail' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-CUST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'customers' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-DATA</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'database_backups' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-INST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'installments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-LEDG</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'ledger' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-PAYM</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'payments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-SALE</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'sales' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-SETT</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'settings' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-SYST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'system_logs' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-USER</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'users' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-AUDI</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'audit_trail' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-CUST</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'customers' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-DATA</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'database_backups' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-INST</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'installments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-LEDG</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'ledger' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-PAYM</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'payments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-SALE</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'sales' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-SETT</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'settings' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-SYST</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'system_logs' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-USER</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'users' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-AUDI</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'audit_trail' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-CUST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'customers' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-DATA</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'database_backups' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-INST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'installments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-LEDG</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'ledger' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-PAYM</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'payments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-SALE</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'sales' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-SETT</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'settings' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-SYST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'system_logs' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-USER</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'users' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-AUDI</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'audit_trail' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-CUST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'customers' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-DATA</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'database_backups' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-INST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'installments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-LEDG</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'ledger' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-PAYM</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'payments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-SALE</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'sales' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-SETT</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'settings' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-SYST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'system_logs' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-USER</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'users' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-001</t>
+  </si>
+  <si>
+    <t>Data Security</t>
+  </si>
+  <si>
+    <t>SSL Certificate Verification</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-002</t>
+  </si>
+  <si>
+    <t>Secure sessions state validation</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-003</t>
+  </si>
+  <si>
+    <t>Verify X-Content-Type-Options: nosniff header present</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-004</t>
+  </si>
+  <si>
+    <t>Verify Clickjacking protection (X-Frame-Options/CSP)</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-005</t>
+  </si>
+  <si>
+    <t>Verify raw password is not stored in localStorage</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-006</t>
+  </si>
+  <si>
+    <t>HSTS Header Compliance Check</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-007</t>
+  </si>
+  <si>
+    <t>Content Security Policy (CSP) presence verification</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-008</t>
+  </si>
+  <si>
+    <t>Referrer-Policy header check</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-009</t>
+  </si>
+  <si>
+    <t>CORS policy validation</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-010</t>
+  </si>
+  <si>
+    <t>Secure/HttpOnly cookie attributes check</t>
+  </si>
+  <si>
     <t>TC-SEC-DEP-001</t>
   </si>
   <si>
@@ -41,93 +482,6 @@
     <t>Check third-party package vulnerabilities</t>
   </si>
   <si>
-    <t>Passed</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-001</t>
-  </si>
-  <si>
-    <t>Access Control</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated read rejection (customers)</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-002</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated write rejection (customers)</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-003</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated read rejection (sales)</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-004</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated write rejection (sales)</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-005</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated write rejection (payments)</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-006</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated write rejection (installments)</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-007</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated write rejection (ledger)</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-015</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated read rejection (payments)</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-016</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated read rejection (installments)</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-017</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated read rejection (ledger)</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-003</t>
-  </si>
-  <si>
-    <t>Data Security</t>
-  </si>
-  <si>
-    <t>Verify X-Content-Type-Options: nosniff header present</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-004</t>
-  </si>
-  <si>
-    <t>Verify Clickjacking protection (X-Frame-Options/CSP)</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-001</t>
-  </si>
-  <si>
-    <t>SSL Certificate Verification</t>
-  </si>
-  <si>
     <t>TC-SEC-VAL-001</t>
   </si>
   <si>
@@ -143,52 +497,10 @@
     <t>Mandatory input validation constraints</t>
   </si>
   <si>
-    <t>TC-SEC-AUTH-008</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated dashboard access block</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-009</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated customers access block</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-010</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated sales access block</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-011</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated payments access block</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-012</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated installments access block</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-013</t>
-  </si>
-  <si>
-    <t>Verify unauthenticated ledger access block</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-014</t>
-  </si>
-  <si>
-    <t>Verify post-login authenticated redirect</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-005</t>
-  </si>
-  <si>
-    <t>Verify raw password is not stored in localStorage</t>
+    <t>TC-SEC-VAL-003</t>
+  </si>
+  <si>
+    <t>SQL Injection boundary input escaping check</t>
   </si>
   <si>
     <t>TC-SEC-VAL-004</t>
@@ -200,40 +512,286 @@
     <t>Verify XSS input validation constraint on phone number</t>
   </si>
   <si>
+    <t>TC-SEC-VAL-005</t>
+  </si>
+  <si>
+    <t>HTML escaping check on Payments input</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-AMT-BOUNDARY</t>
+  </si>
+  <si>
+    <t>Verify Boundary validation check on Payment Amount</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-AMT-EMPTY</t>
+  </si>
+  <si>
+    <t>Verify Null/Empty input constraint on Payment Amount</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-AMT-FORMAT</t>
+  </si>
+  <si>
+    <t>Verify Format conformity audit on Payment Amount</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-AMT-OVERFLOW</t>
+  </si>
+  <si>
+    <t>Verify Character limit overflow check on Payment Amount</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-AMT-SPECIAL</t>
+  </si>
+  <si>
+    <t>Verify Special character sanitation on Payment Amount</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-DATE-BOUNDARY</t>
+  </si>
+  <si>
+    <t>Verify Boundary validation check on Transaction Date</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-DATE-EMPTY</t>
+  </si>
+  <si>
+    <t>Verify Null/Empty input constraint on Transaction Date</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-DATE-FORMAT</t>
+  </si>
+  <si>
+    <t>Verify Format conformity audit on Transaction Date</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-DATE-OVERFLOW</t>
+  </si>
+  <si>
+    <t>Verify Character limit overflow check on Transaction Date</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-DATE-SPECIAL</t>
+  </si>
+  <si>
+    <t>Verify Special character sanitation on Transaction Date</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-EMAIL-BOUNDARY</t>
+  </si>
+  <si>
+    <t>Verify Boundary validation check on Email Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-EMAIL-EMPTY</t>
+  </si>
+  <si>
+    <t>Verify Null/Empty input constraint on Email Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-EMAIL-FORMAT</t>
+  </si>
+  <si>
+    <t>Verify Format conformity audit on Email Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-EMAIL-OVERFLOW</t>
+  </si>
+  <si>
+    <t>Verify Character limit overflow check on Email Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-EMAIL-SPECIAL</t>
+  </si>
+  <si>
+    <t>Verify Special character sanitation on Email Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PASS-BOUNDARY</t>
+  </si>
+  <si>
+    <t>Verify Boundary validation check on Password Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PASS-EMPTY</t>
+  </si>
+  <si>
+    <t>Verify Null/Empty input constraint on Password Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PASS-FORMAT</t>
+  </si>
+  <si>
+    <t>Verify Format conformity audit on Password Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PASS-OVERFLOW</t>
+  </si>
+  <si>
+    <t>Verify Character limit overflow check on Password Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PASS-SPECIAL</t>
+  </si>
+  <si>
+    <t>Verify Special character sanitation on Password Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PHONE-BOUNDARY</t>
+  </si>
+  <si>
+    <t>Verify Boundary validation check on Phone Number</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PHONE-EMPTY</t>
+  </si>
+  <si>
+    <t>Verify Null/Empty input constraint on Phone Number</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PHONE-FORMAT</t>
+  </si>
+  <si>
+    <t>Verify Format conformity audit on Phone Number</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PHONE-OVERFLOW</t>
+  </si>
+  <si>
+    <t>Verify Character limit overflow check on Phone Number</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PHONE-SPECIAL</t>
+  </si>
+  <si>
+    <t>Verify Special character sanitation on Phone Number</t>
+  </si>
+  <si>
     <t>TC-SEC-XSS-001</t>
   </si>
   <si>
     <t>XSS escaping on Customer creation name field</t>
   </si>
   <si>
-    <t>TC-SEC-XSS-002</t>
-  </si>
-  <si>
-    <t>XSS escaping on Sales creation</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-003</t>
-  </si>
-  <si>
-    <t>SQL Injection boundary input escaping check</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-005</t>
-  </si>
-  <si>
-    <t>HTML escaping check on Payments input</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-002</t>
-  </si>
-  <si>
-    <t>Secure sessions state validation</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-018</t>
-  </si>
-  <si>
-    <t>Verify session termination and login redirect on logout</t>
+    <t>TC-SEC-XSS-ITEM-001</t>
+  </si>
+  <si>
+    <t>Verify protection against Script tag injection on Sale Item Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-ITEM-002</t>
+  </si>
+  <si>
+    <t>Verify protection against Image error handler attribute on Sale Item Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-ITEM-003</t>
+  </si>
+  <si>
+    <t>Verify protection against SVG onload handler on Sale Item Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-ITEM-004</t>
+  </si>
+  <si>
+    <t>Verify protection against Javascript protocol URI on Sale Item Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-ITEM-005</t>
+  </si>
+  <si>
+    <t>Verify protection against Iframe source injection on Sale Item Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-NAME-001</t>
+  </si>
+  <si>
+    <t>Verify protection against Script tag injection on Customer Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-NAME-002</t>
+  </si>
+  <si>
+    <t>Verify protection against Image error handler attribute on Customer Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-NAME-003</t>
+  </si>
+  <si>
+    <t>Verify protection against SVG onload handler on Customer Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-NAME-004</t>
+  </si>
+  <si>
+    <t>Verify protection against Javascript protocol URI on Customer Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-NAME-005</t>
+  </si>
+  <si>
+    <t>Verify protection against Iframe source injection on Customer Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-PROF-001</t>
+  </si>
+  <si>
+    <t>Verify protection against Script tag injection on User Profile Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-PROF-002</t>
+  </si>
+  <si>
+    <t>Verify protection against Image error handler attribute on User Profile Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-PROF-003</t>
+  </si>
+  <si>
+    <t>Verify protection against SVG onload handler on User Profile Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-PROF-004</t>
+  </si>
+  <si>
+    <t>Verify protection against Javascript protocol URI on User Profile Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-PROF-005</t>
+  </si>
+  <si>
+    <t>Verify protection against Iframe source injection on User Profile Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-REM-001</t>
+  </si>
+  <si>
+    <t>Verify protection against Script tag injection on Payment Remarks</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-REM-002</t>
+  </si>
+  <si>
+    <t>Verify protection against Image error handler attribute on Payment Remarks</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-REM-003</t>
+  </si>
+  <si>
+    <t>Verify protection against SVG onload handler on Payment Remarks</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-REM-004</t>
+  </si>
+  <si>
+    <t>Verify protection against Javascript protocol URI on Payment Remarks</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-REM-005</t>
+  </si>
+  <si>
+    <t>Verify protection against Iframe source injection on Payment Remarks</t>
   </si>
   <si>
     <t>PAYBUDDY WEB SECURITY REPORT</t>
@@ -794,7 +1352,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D128"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="60" customWidth="1"/>
@@ -849,10 +1407,10 @@
         <v>10</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>11</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>12</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>9</v>
@@ -860,13 +1418,13 @@
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>13</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>14</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>9</v>
@@ -874,13 +1432,13 @@
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>16</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>9</v>
@@ -888,13 +1446,13 @@
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>18</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>9</v>
@@ -902,13 +1460,13 @@
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>19</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>20</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>9</v>
@@ -916,13 +1474,13 @@
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>21</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>22</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>9</v>
@@ -930,13 +1488,13 @@
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>23</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>24</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>9</v>
@@ -944,13 +1502,13 @@
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>26</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>9</v>
@@ -958,13 +1516,13 @@
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>28</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>9</v>
@@ -972,13 +1530,13 @@
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>30</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>9</v>
@@ -986,13 +1544,13 @@
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>33</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>9</v>
@@ -1000,13 +1558,13 @@
     </row>
     <row r="17" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>9</v>
@@ -1014,13 +1572,13 @@
     </row>
     <row r="18" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>9</v>
@@ -1028,13 +1586,13 @@
     </row>
     <row r="19" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>9</v>
@@ -1042,13 +1600,13 @@
     </row>
     <row r="20" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B20" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>42</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>9</v>
@@ -1056,13 +1614,13 @@
     </row>
     <row r="21" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>9</v>
@@ -1070,13 +1628,13 @@
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>9</v>
@@ -1084,13 +1642,13 @@
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>9</v>
@@ -1098,13 +1656,13 @@
     </row>
     <row r="24" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>9</v>
@@ -1112,13 +1670,13 @@
     </row>
     <row r="25" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>9</v>
@@ -1126,13 +1684,13 @@
     </row>
     <row r="26" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>9</v>
@@ -1140,13 +1698,13 @@
     </row>
     <row r="27" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>9</v>
@@ -1154,13 +1712,13 @@
     </row>
     <row r="28" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>9</v>
@@ -1168,13 +1726,13 @@
     </row>
     <row r="29" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>60</v>
+        <v>7</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>9</v>
@@ -1182,13 +1740,13 @@
     </row>
     <row r="30" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>60</v>
+        <v>7</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>9</v>
@@ -1196,13 +1754,13 @@
     </row>
     <row r="31" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>60</v>
+        <v>7</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>9</v>
@@ -1210,13 +1768,13 @@
     </row>
     <row r="32" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>9</v>
@@ -1224,13 +1782,13 @@
     </row>
     <row r="33" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>9</v>
@@ -1238,13 +1796,13 @@
     </row>
     <row r="34" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>9</v>
@@ -1252,15 +1810,1317 @@
     </row>
     <row r="35" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B35" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C35" s="4" t="s">
+      <c r="B37" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="D37" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D61" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="D62" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D63" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D65" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D66" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="D67" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D68" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D70" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D71" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D73" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D76" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D77" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="D78" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="D79" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D80" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D81" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D82" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="D83" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="D84" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="D85" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="D86" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="D87" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="D88" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="D89" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="D90" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="D91" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="D92" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="D93" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="D94" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="D95" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="D96" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="D97" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="D99" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="D100" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="D101" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C102" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="D102" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A103" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="D103" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A104" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C104" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="D104" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="D105" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A106" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C106" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="D106" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A107" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="D107" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A108" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C108" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="D108" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A109" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="D109" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A110" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C110" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="D110" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A111" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="D111" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A112" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="D112" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A113" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="D113" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A115" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C115" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="D115" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C116" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="D116" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A117" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C117" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="D117" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A118" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C118" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="D118" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A119" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C119" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D119" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A120" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C120" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="D120" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A121" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C121" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="D121" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A122" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C122" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="D122" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C123" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="D123" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A124" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C124" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="D124" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A125" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="D125" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="126" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A126" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C126" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="127" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A127" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="128" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A128" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="D128" s="5" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1285,33 +3145,33 @@
   <sheetData>
     <row r="1" ht="35" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>74</v>
+        <v>260</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>75</v>
+        <v>261</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>76</v>
+        <v>262</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>77</v>
+        <v>263</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>78</v>
+        <v>264</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>79</v>
+        <v>265</v>
       </c>
       <c r="B6" s="11">
-        <v>31</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -1319,12 +3179,12 @@
         <v>9</v>
       </c>
       <c r="B7" s="5">
-        <v>31</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>80</v>
+        <v>266</v>
       </c>
       <c r="B8" s="11">
         <v>0</v>
@@ -1332,7 +3192,7 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>81</v>
+        <v>267</v>
       </c>
       <c r="B9" s="11">
         <v>0</v>
@@ -1340,18 +3200,18 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>82</v>
+        <v>268</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>83</v>
+        <v>269</v>
       </c>
     </row>
     <row r="12" ht="25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>84</v>
+        <v>270</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>85</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: add support for GITHUB_STEP_SUMMARY in E2E, security, and load tests
</commit_message>
<xml_diff>
--- a/tests/reports/Vulnerability_Analysis_Report.xlsx
+++ b/tests/reports/Vulnerability_Analysis_Report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="306">
   <si>
     <t>PAYBUDDY WEB SECURITY REPORT</t>
   </si>
@@ -20,7 +20,7 @@
     <t>Scan Date</t>
   </si>
   <si>
-    <t>22-Jun-2026</t>
+    <t>25-Jun-2026</t>
   </si>
   <si>
     <t>Metric</t>
@@ -56,7 +56,7 @@
     <t>PAYBUDDY SECURITY &amp; VULNERABILITY ANALYSIS REPORT</t>
   </si>
   <si>
-    <t>Generated: 22/6/2026, 3:41:10 pm | Scans Completed: 124 | Status: SECURE</t>
+    <t>Generated: 25/6/2026, 11:47:38 am | Scans Completed: 124 | Status: SECURE</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -83,820 +83,811 @@
     <t>Verify post-login authenticated redirect</t>
   </si>
   <si>
+    <t>27ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-018</t>
+  </si>
+  <si>
+    <t>Verify session termination and login redirect on logout</t>
+  </si>
+  <si>
+    <t>16ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-AUDI</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'audit_trail' collection</t>
+  </si>
+  <si>
+    <t>14ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-CUST</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'customers' collection</t>
+  </si>
+  <si>
+    <t>21ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-DATA</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'database_backups' collection</t>
+  </si>
+  <si>
+    <t>37ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-INST</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'installments' collection</t>
+  </si>
+  <si>
+    <t>32ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-LEDG</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'ledger' collection</t>
+  </si>
+  <si>
+    <t>24ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-PAYM</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'payments' collection</t>
+  </si>
+  <si>
+    <t>33ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-SALE</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'sales' collection</t>
+  </si>
+  <si>
+    <t>28ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-SETT</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'settings' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-SYST</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'system_logs' collection</t>
+  </si>
+  <si>
+    <t>31ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-B-USER</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Batch Read Rejection on 'users' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-AUDI</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'audit_trail' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-CUST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'customers' collection</t>
+  </si>
+  <si>
+    <t>29ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-DATA</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'database_backups' collection</t>
+  </si>
+  <si>
+    <t>26ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-INST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'installments' collection</t>
+  </si>
+  <si>
+    <t>23ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-LEDG</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'ledger' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-PAYM</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'payments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-SALE</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'sales' collection</t>
+  </si>
+  <si>
     <t>13ms</t>
   </si>
   <si>
-    <t>TC-SEC-AUTH-018</t>
-  </si>
-  <si>
-    <t>Verify session termination and login redirect on logout</t>
-  </si>
-  <si>
-    <t>29ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-B-AUDI</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Batch Read Rejection on 'audit_trail' collection</t>
+    <t>TC-SEC-AUTH-D-SETT</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'settings' collection</t>
+  </si>
+  <si>
+    <t>20ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-SYST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'system_logs' collection</t>
+  </si>
+  <si>
+    <t>36ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-D-USER</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Delete Rejection on 'users' collection</t>
   </si>
   <si>
     <t>35ms</t>
   </si>
   <si>
-    <t>TC-SEC-AUTH-B-CUST</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Batch Read Rejection on 'customers' collection</t>
-  </si>
-  <si>
-    <t>37ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-B-DATA</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Batch Read Rejection on 'database_backups' collection</t>
-  </si>
-  <si>
-    <t>16ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-B-INST</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Batch Read Rejection on 'installments' collection</t>
-  </si>
-  <si>
-    <t>23ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-B-LEDG</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Batch Read Rejection on 'ledger' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-B-PAYM</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Batch Read Rejection on 'payments' collection</t>
-  </si>
-  <si>
-    <t>20ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-B-SALE</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Batch Read Rejection on 'sales' collection</t>
+    <t>TC-SEC-AUTH-R-AUDI</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'audit_trail' collection</t>
+  </si>
+  <si>
+    <t>12ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-CUST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'customers' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-DATA</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'database_backups' collection</t>
+  </si>
+  <si>
+    <t>22ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-INST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'installments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-LEDG</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'ledger' collection</t>
+  </si>
+  <si>
+    <t>34ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-PAYM</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'payments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-SALE</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'sales' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-SETT</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'settings' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-SYST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'system_logs' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-R-USER</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Read Rejection on 'users' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-AUDI</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'audit_trail' collection</t>
+  </si>
+  <si>
+    <t>38ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-CUST</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'customers' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-DATA</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'database_backups' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-INST</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'installments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-LEDG</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'ledger' collection</t>
+  </si>
+  <si>
+    <t>15ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-PAYM</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'payments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-SALE</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'sales' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-SETT</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'settings' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-SYST</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'system_logs' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-S-USER</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Schema Mutation Rejection on 'users' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-AUDI</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'audit_trail' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-CUST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'customers' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-DATA</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'database_backups' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-INST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'installments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-LEDG</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'ledger' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-PAYM</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'payments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-SALE</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'sales' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-SETT</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'settings' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-SYST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'system_logs' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-U-USER</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Update Rejection on 'users' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-AUDI</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'audit_trail' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-CUST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'customers' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-DATA</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'database_backups' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-INST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'installments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-LEDG</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'ledger' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-PAYM</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'payments' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-SALE</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'sales' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-SETT</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'settings' collection</t>
+  </si>
+  <si>
+    <t>25ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-SYST</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'system_logs' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-AUTH-W-USER</t>
+  </si>
+  <si>
+    <t>Verify Unauthenticated Write Rejection on 'users' collection</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-001</t>
+  </si>
+  <si>
+    <t>Data Security</t>
+  </si>
+  <si>
+    <t>SSL Certificate Verification</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-002</t>
+  </si>
+  <si>
+    <t>Secure sessions state validation</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-003</t>
+  </si>
+  <si>
+    <t>Verify X-Content-Type-Options: nosniff header present</t>
+  </si>
+  <si>
+    <t>53ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-004</t>
+  </si>
+  <si>
+    <t>Verify Clickjacking protection (X-Frame-Options/CSP)</t>
+  </si>
+  <si>
+    <t>52ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-005</t>
+  </si>
+  <si>
+    <t>Verify raw password is not stored in localStorage</t>
+  </si>
+  <si>
+    <t>47ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-006</t>
+  </si>
+  <si>
+    <t>HSTS Header Compliance Check</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-007</t>
+  </si>
+  <si>
+    <t>Content Security Policy (CSP) presence verification</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-008</t>
+  </si>
+  <si>
+    <t>Referrer-Policy header check</t>
+  </si>
+  <si>
+    <t>43ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-009</t>
+  </si>
+  <si>
+    <t>CORS policy validation</t>
+  </si>
+  <si>
+    <t>TC-SEC-CONF-010</t>
+  </si>
+  <si>
+    <t>Secure/HttpOnly cookie attributes check</t>
+  </si>
+  <si>
+    <t>58ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-DEP-001</t>
+  </si>
+  <si>
+    <t>Dependency Audit</t>
+  </si>
+  <si>
+    <t>Check third-party package vulnerabilities</t>
+  </si>
+  <si>
+    <t>382ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-001</t>
+  </si>
+  <si>
+    <t>Input Validation</t>
+  </si>
+  <si>
+    <t>Password masking verification</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-002</t>
+  </si>
+  <si>
+    <t>Mandatory input validation constraints</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-003</t>
+  </si>
+  <si>
+    <t>SQL Injection boundary input escaping check</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-004</t>
+  </si>
+  <si>
+    <t>XSS Prevention</t>
+  </si>
+  <si>
+    <t>Verify XSS input validation constraint on phone number</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-005</t>
+  </si>
+  <si>
+    <t>HTML escaping check on Payments input</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-AMT-BOUNDARY</t>
+  </si>
+  <si>
+    <t>Verify Boundary validation check on Payment Amount</t>
   </si>
   <si>
     <t>18ms</t>
   </si>
   <si>
-    <t>TC-SEC-AUTH-B-SETT</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Batch Read Rejection on 'settings' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-B-SYST</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Batch Read Rejection on 'system_logs' collection</t>
-  </si>
-  <si>
-    <t>30ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-B-USER</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Batch Read Rejection on 'users' collection</t>
-  </si>
-  <si>
-    <t>21ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-D-AUDI</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Delete Rejection on 'audit_trail' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-D-CUST</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Delete Rejection on 'customers' collection</t>
-  </si>
-  <si>
-    <t>36ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-D-DATA</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Delete Rejection on 'database_backups' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-D-INST</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Delete Rejection on 'installments' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-D-LEDG</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Delete Rejection on 'ledger' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-D-PAYM</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Delete Rejection on 'payments' collection</t>
-  </si>
-  <si>
-    <t>22ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-D-SALE</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Delete Rejection on 'sales' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-D-SETT</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Delete Rejection on 'settings' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-D-SYST</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Delete Rejection on 'system_logs' collection</t>
+    <t>TC-SEC-VAL-AMT-EMPTY</t>
+  </si>
+  <si>
+    <t>Verify Null/Empty input constraint on Payment Amount</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-AMT-FORMAT</t>
+  </si>
+  <si>
+    <t>Verify Format conformity audit on Payment Amount</t>
+  </si>
+  <si>
+    <t>8ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-AMT-OVERFLOW</t>
+  </si>
+  <si>
+    <t>Verify Character limit overflow check on Payment Amount</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-AMT-SPECIAL</t>
+  </si>
+  <si>
+    <t>Verify Special character sanitation on Payment Amount</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-DATE-BOUNDARY</t>
+  </si>
+  <si>
+    <t>Verify Boundary validation check on Transaction Date</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-DATE-EMPTY</t>
+  </si>
+  <si>
+    <t>Verify Null/Empty input constraint on Transaction Date</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-DATE-FORMAT</t>
+  </si>
+  <si>
+    <t>Verify Format conformity audit on Transaction Date</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-DATE-OVERFLOW</t>
+  </si>
+  <si>
+    <t>Verify Character limit overflow check on Transaction Date</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-DATE-SPECIAL</t>
+  </si>
+  <si>
+    <t>Verify Special character sanitation on Transaction Date</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-EMAIL-BOUNDARY</t>
+  </si>
+  <si>
+    <t>Verify Boundary validation check on Email Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-EMAIL-EMPTY</t>
+  </si>
+  <si>
+    <t>Verify Null/Empty input constraint on Email Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-EMAIL-FORMAT</t>
+  </si>
+  <si>
+    <t>Verify Format conformity audit on Email Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-EMAIL-OVERFLOW</t>
+  </si>
+  <si>
+    <t>Verify Character limit overflow check on Email Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-EMAIL-SPECIAL</t>
+  </si>
+  <si>
+    <t>Verify Special character sanitation on Email Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PASS-BOUNDARY</t>
+  </si>
+  <si>
+    <t>Verify Boundary validation check on Password Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PASS-EMPTY</t>
+  </si>
+  <si>
+    <t>Verify Null/Empty input constraint on Password Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PASS-FORMAT</t>
+  </si>
+  <si>
+    <t>Verify Format conformity audit on Password Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PASS-OVERFLOW</t>
+  </si>
+  <si>
+    <t>Verify Character limit overflow check on Password Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PASS-SPECIAL</t>
+  </si>
+  <si>
+    <t>Verify Special character sanitation on Password Field</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PHONE-BOUNDARY</t>
+  </si>
+  <si>
+    <t>Verify Boundary validation check on Phone Number</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PHONE-EMPTY</t>
+  </si>
+  <si>
+    <t>Verify Null/Empty input constraint on Phone Number</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PHONE-FORMAT</t>
+  </si>
+  <si>
+    <t>Verify Format conformity audit on Phone Number</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PHONE-OVERFLOW</t>
+  </si>
+  <si>
+    <t>Verify Character limit overflow check on Phone Number</t>
+  </si>
+  <si>
+    <t>TC-SEC-VAL-PHONE-SPECIAL</t>
+  </si>
+  <si>
+    <t>Verify Special character sanitation on Phone Number</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-001</t>
+  </si>
+  <si>
+    <t>XSS escaping on Customer creation name field</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-ITEM-001</t>
+  </si>
+  <si>
+    <t>Verify protection against Script tag injection on Sale Item Name</t>
+  </si>
+  <si>
+    <t>19ms</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-ITEM-002</t>
+  </si>
+  <si>
+    <t>Verify protection against Image error handler attribute on Sale Item Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-ITEM-003</t>
+  </si>
+  <si>
+    <t>Verify protection against SVG onload handler on Sale Item Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-ITEM-004</t>
+  </si>
+  <si>
+    <t>Verify protection against Javascript protocol URI on Sale Item Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-ITEM-005</t>
+  </si>
+  <si>
+    <t>Verify protection against Iframe source injection on Sale Item Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-NAME-001</t>
+  </si>
+  <si>
+    <t>Verify protection against Script tag injection on Customer Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-NAME-002</t>
+  </si>
+  <si>
+    <t>Verify protection against Image error handler attribute on Customer Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-NAME-003</t>
+  </si>
+  <si>
+    <t>Verify protection against SVG onload handler on Customer Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-NAME-004</t>
+  </si>
+  <si>
+    <t>Verify protection against Javascript protocol URI on Customer Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-NAME-005</t>
+  </si>
+  <si>
+    <t>Verify protection against Iframe source injection on Customer Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-PROF-001</t>
+  </si>
+  <si>
+    <t>Verify protection against Script tag injection on User Profile Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-PROF-002</t>
+  </si>
+  <si>
+    <t>Verify protection against Image error handler attribute on User Profile Name</t>
+  </si>
+  <si>
+    <t>TC-SEC-XSS-PROF-003</t>
+  </si>
+  <si>
+    <t>Verify protection against SVG onload handler on User Profile Name</t>
   </si>
   <si>
     <t>17ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-D-USER</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Delete Rejection on 'users' collection</t>
-  </si>
-  <si>
-    <t>24ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-R-AUDI</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Read Rejection on 'audit_trail' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-R-CUST</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Read Rejection on 'customers' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-R-DATA</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Read Rejection on 'database_backups' collection</t>
-  </si>
-  <si>
-    <t>27ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-R-INST</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Read Rejection on 'installments' collection</t>
-  </si>
-  <si>
-    <t>19ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-R-LEDG</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Read Rejection on 'ledger' collection</t>
-  </si>
-  <si>
-    <t>14ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-R-PAYM</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Read Rejection on 'payments' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-R-SALE</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Read Rejection on 'sales' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-R-SETT</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Read Rejection on 'settings' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-R-SYST</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Read Rejection on 'system_logs' collection</t>
-  </si>
-  <si>
-    <t>15ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-R-USER</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Read Rejection on 'users' collection</t>
-  </si>
-  <si>
-    <t>25ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-S-AUDI</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Schema Mutation Rejection on 'audit_trail' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-S-CUST</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Schema Mutation Rejection on 'customers' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-S-DATA</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Schema Mutation Rejection on 'database_backups' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-S-INST</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Schema Mutation Rejection on 'installments' collection</t>
-  </si>
-  <si>
-    <t>26ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-S-LEDG</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Schema Mutation Rejection on 'ledger' collection</t>
-  </si>
-  <si>
-    <t>39ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-S-PAYM</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Schema Mutation Rejection on 'payments' collection</t>
-  </si>
-  <si>
-    <t>28ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-S-SALE</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Schema Mutation Rejection on 'sales' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-S-SETT</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Schema Mutation Rejection on 'settings' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-S-SYST</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Schema Mutation Rejection on 'system_logs' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-S-USER</t>
-  </si>
-  <si>
-    <t>Verify Unauthorized Schema Mutation Rejection on 'users' collection</t>
-  </si>
-  <si>
-    <t>38ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-U-AUDI</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Update Rejection on 'audit_trail' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-U-CUST</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Update Rejection on 'customers' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-U-DATA</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Update Rejection on 'database_backups' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-U-INST</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Update Rejection on 'installments' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-U-LEDG</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Update Rejection on 'ledger' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-U-PAYM</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Update Rejection on 'payments' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-U-SALE</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Update Rejection on 'sales' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-U-SETT</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Update Rejection on 'settings' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-U-SYST</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Update Rejection on 'system_logs' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-U-USER</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Update Rejection on 'users' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-W-AUDI</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Write Rejection on 'audit_trail' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-W-CUST</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Write Rejection on 'customers' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-W-DATA</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Write Rejection on 'database_backups' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-W-INST</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Write Rejection on 'installments' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-W-LEDG</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Write Rejection on 'ledger' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-W-PAYM</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Write Rejection on 'payments' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-W-SALE</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Write Rejection on 'sales' collection</t>
-  </si>
-  <si>
-    <t>34ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-W-SETT</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Write Rejection on 'settings' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-W-SYST</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Write Rejection on 'system_logs' collection</t>
-  </si>
-  <si>
-    <t>TC-SEC-AUTH-W-USER</t>
-  </si>
-  <si>
-    <t>Verify Unauthenticated Write Rejection on 'users' collection</t>
-  </si>
-  <si>
-    <t>31ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-001</t>
-  </si>
-  <si>
-    <t>Data Security</t>
-  </si>
-  <si>
-    <t>SSL Certificate Verification</t>
-  </si>
-  <si>
-    <t>43ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-002</t>
-  </si>
-  <si>
-    <t>Secure sessions state validation</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-003</t>
-  </si>
-  <si>
-    <t>Verify X-Content-Type-Options: nosniff header present</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-004</t>
-  </si>
-  <si>
-    <t>Verify Clickjacking protection (X-Frame-Options/CSP)</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-005</t>
-  </si>
-  <si>
-    <t>Verify raw password is not stored in localStorage</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-006</t>
-  </si>
-  <si>
-    <t>HSTS Header Compliance Check</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-007</t>
-  </si>
-  <si>
-    <t>Content Security Policy (CSP) presence verification</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-008</t>
-  </si>
-  <si>
-    <t>Referrer-Policy header check</t>
-  </si>
-  <si>
-    <t>40ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-009</t>
-  </si>
-  <si>
-    <t>CORS policy validation</t>
-  </si>
-  <si>
-    <t>55ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-CONF-010</t>
-  </si>
-  <si>
-    <t>Secure/HttpOnly cookie attributes check</t>
-  </si>
-  <si>
-    <t>49ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-DEP-001</t>
-  </si>
-  <si>
-    <t>Dependency Audit</t>
-  </si>
-  <si>
-    <t>Check third-party package vulnerabilities</t>
-  </si>
-  <si>
-    <t>569ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-001</t>
-  </si>
-  <si>
-    <t>Input Validation</t>
-  </si>
-  <si>
-    <t>Password masking verification</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-002</t>
-  </si>
-  <si>
-    <t>Mandatory input validation constraints</t>
-  </si>
-  <si>
-    <t>8ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-003</t>
-  </si>
-  <si>
-    <t>SQL Injection boundary input escaping check</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-004</t>
-  </si>
-  <si>
-    <t>XSS Prevention</t>
-  </si>
-  <si>
-    <t>Verify XSS input validation constraint on phone number</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-005</t>
-  </si>
-  <si>
-    <t>HTML escaping check on Payments input</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-AMT-BOUNDARY</t>
-  </si>
-  <si>
-    <t>Verify Boundary validation check on Payment Amount</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-AMT-EMPTY</t>
-  </si>
-  <si>
-    <t>Verify Null/Empty input constraint on Payment Amount</t>
-  </si>
-  <si>
-    <t>10ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-AMT-FORMAT</t>
-  </si>
-  <si>
-    <t>Verify Format conformity audit on Payment Amount</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-AMT-OVERFLOW</t>
-  </si>
-  <si>
-    <t>Verify Character limit overflow check on Payment Amount</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-AMT-SPECIAL</t>
-  </si>
-  <si>
-    <t>Verify Special character sanitation on Payment Amount</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-DATE-BOUNDARY</t>
-  </si>
-  <si>
-    <t>Verify Boundary validation check on Transaction Date</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-DATE-EMPTY</t>
-  </si>
-  <si>
-    <t>Verify Null/Empty input constraint on Transaction Date</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-DATE-FORMAT</t>
-  </si>
-  <si>
-    <t>Verify Format conformity audit on Transaction Date</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-DATE-OVERFLOW</t>
-  </si>
-  <si>
-    <t>Verify Character limit overflow check on Transaction Date</t>
-  </si>
-  <si>
-    <t>11ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-DATE-SPECIAL</t>
-  </si>
-  <si>
-    <t>Verify Special character sanitation on Transaction Date</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-EMAIL-BOUNDARY</t>
-  </si>
-  <si>
-    <t>Verify Boundary validation check on Email Field</t>
-  </si>
-  <si>
-    <t>9ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-EMAIL-EMPTY</t>
-  </si>
-  <si>
-    <t>Verify Null/Empty input constraint on Email Field</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-EMAIL-FORMAT</t>
-  </si>
-  <si>
-    <t>Verify Format conformity audit on Email Field</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-EMAIL-OVERFLOW</t>
-  </si>
-  <si>
-    <t>Verify Character limit overflow check on Email Field</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-EMAIL-SPECIAL</t>
-  </si>
-  <si>
-    <t>Verify Special character sanitation on Email Field</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-PASS-BOUNDARY</t>
-  </si>
-  <si>
-    <t>Verify Boundary validation check on Password Field</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-PASS-EMPTY</t>
-  </si>
-  <si>
-    <t>Verify Null/Empty input constraint on Password Field</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-PASS-FORMAT</t>
-  </si>
-  <si>
-    <t>Verify Format conformity audit on Password Field</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-PASS-OVERFLOW</t>
-  </si>
-  <si>
-    <t>Verify Character limit overflow check on Password Field</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-PASS-SPECIAL</t>
-  </si>
-  <si>
-    <t>Verify Special character sanitation on Password Field</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-PHONE-BOUNDARY</t>
-  </si>
-  <si>
-    <t>Verify Boundary validation check on Phone Number</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-PHONE-EMPTY</t>
-  </si>
-  <si>
-    <t>Verify Null/Empty input constraint on Phone Number</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-PHONE-FORMAT</t>
-  </si>
-  <si>
-    <t>Verify Format conformity audit on Phone Number</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-PHONE-OVERFLOW</t>
-  </si>
-  <si>
-    <t>Verify Character limit overflow check on Phone Number</t>
-  </si>
-  <si>
-    <t>TC-SEC-VAL-PHONE-SPECIAL</t>
-  </si>
-  <si>
-    <t>Verify Special character sanitation on Phone Number</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-001</t>
-  </si>
-  <si>
-    <t>XSS escaping on Customer creation name field</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-ITEM-001</t>
-  </si>
-  <si>
-    <t>Verify protection against Script tag injection on Sale Item Name</t>
-  </si>
-  <si>
-    <t>32ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-ITEM-002</t>
-  </si>
-  <si>
-    <t>Verify protection against Image error handler attribute on Sale Item Name</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-ITEM-003</t>
-  </si>
-  <si>
-    <t>Verify protection against SVG onload handler on Sale Item Name</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-ITEM-004</t>
-  </si>
-  <si>
-    <t>Verify protection against Javascript protocol URI on Sale Item Name</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-ITEM-005</t>
-  </si>
-  <si>
-    <t>Verify protection against Iframe source injection on Sale Item Name</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-NAME-001</t>
-  </si>
-  <si>
-    <t>Verify protection against Script tag injection on Customer Name</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-NAME-002</t>
-  </si>
-  <si>
-    <t>Verify protection against Image error handler attribute on Customer Name</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-NAME-003</t>
-  </si>
-  <si>
-    <t>Verify protection against SVG onload handler on Customer Name</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-NAME-004</t>
-  </si>
-  <si>
-    <t>Verify protection against Javascript protocol URI on Customer Name</t>
-  </si>
-  <si>
-    <t>33ms</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-NAME-005</t>
-  </si>
-  <si>
-    <t>Verify protection against Iframe source injection on Customer Name</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-PROF-001</t>
-  </si>
-  <si>
-    <t>Verify protection against Script tag injection on User Profile Name</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-PROF-002</t>
-  </si>
-  <si>
-    <t>Verify protection against Image error handler attribute on User Profile Name</t>
-  </si>
-  <si>
-    <t>TC-SEC-XSS-PROF-003</t>
-  </si>
-  <si>
-    <t>Verify protection against SVG onload handler on User Profile Name</t>
   </si>
   <si>
     <t>TC-SEC-XSS-PROF-004</t>
@@ -1706,7 +1697,7 @@
         <v>40</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>6</v>
@@ -1714,16 +1705,16 @@
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B12" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>6</v>
@@ -1731,16 +1722,16 @@
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B13" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>6</v>
@@ -1748,16 +1739,16 @@
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B14" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>6</v>
@@ -1765,16 +1756,16 @@
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B15" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>6</v>
@@ -1782,16 +1773,16 @@
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B16" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>6</v>
@@ -1808,7 +1799,7 @@
         <v>56</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>6</v>
@@ -1842,7 +1833,7 @@
         <v>61</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>6</v>
@@ -1850,16 +1841,16 @@
     </row>
     <row r="20" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B20" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="E20" s="7" t="s">
         <v>6</v>
@@ -1867,16 +1858,16 @@
     </row>
     <row r="21" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B21" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="E21" s="7" t="s">
         <v>6</v>
@@ -1884,16 +1875,16 @@
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B22" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>6</v>
@@ -1901,16 +1892,16 @@
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B23" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>46</v>
+        <v>72</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>6</v>
@@ -1918,16 +1909,16 @@
     </row>
     <row r="24" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B24" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>6</v>
@@ -1935,16 +1926,16 @@
     </row>
     <row r="25" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B25" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>6</v>
@@ -1952,16 +1943,16 @@
     </row>
     <row r="26" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B26" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>6</v>
@@ -1969,16 +1960,16 @@
     </row>
     <row r="27" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B27" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>43</v>
+        <v>84</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>6</v>
@@ -1986,16 +1977,16 @@
     </row>
     <row r="28" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B28" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E28" s="7" t="s">
         <v>6</v>
@@ -2003,16 +1994,16 @@
     </row>
     <row r="29" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B29" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="E29" s="7" t="s">
         <v>6</v>
@@ -2020,16 +2011,16 @@
     </row>
     <row r="30" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B30" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="E30" s="7" t="s">
         <v>6</v>
@@ -2037,16 +2028,16 @@
     </row>
     <row r="31" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B31" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="E31" s="7" t="s">
         <v>6</v>
@@ -2054,16 +2045,16 @@
     </row>
     <row r="32" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B32" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E32" s="7" t="s">
         <v>6</v>
@@ -2071,16 +2062,16 @@
     </row>
     <row r="33" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="D33" s="13" t="s">
         <v>94</v>
-      </c>
-      <c r="B33" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="D33" s="13" t="s">
-        <v>26</v>
       </c>
       <c r="E33" s="7" t="s">
         <v>6</v>
@@ -2088,16 +2079,16 @@
     </row>
     <row r="34" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B34" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>6</v>
@@ -2105,16 +2096,16 @@
     </row>
     <row r="35" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="13" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B35" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>6</v>
@@ -2122,16 +2113,16 @@
     </row>
     <row r="36" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B36" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>6</v>
@@ -2139,16 +2130,16 @@
     </row>
     <row r="37" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B37" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>78</v>
+        <v>107</v>
       </c>
       <c r="E37" s="7" t="s">
         <v>6</v>
@@ -2156,16 +2147,16 @@
     </row>
     <row r="38" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="13" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B38" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="E38" s="7" t="s">
         <v>6</v>
@@ -2173,16 +2164,16 @@
     </row>
     <row r="39" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="13" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B39" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="E39" s="7" t="s">
         <v>6</v>
@@ -2190,16 +2181,16 @@
     </row>
     <row r="40" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B40" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>112</v>
+        <v>84</v>
       </c>
       <c r="E40" s="7" t="s">
         <v>6</v>
@@ -2207,16 +2198,16 @@
     </row>
     <row r="41" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B41" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E41" s="7" t="s">
         <v>6</v>
@@ -2224,16 +2215,16 @@
     </row>
     <row r="42" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="13" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B42" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>118</v>
+        <v>23</v>
       </c>
       <c r="E42" s="7" t="s">
         <v>6</v>
@@ -2250,7 +2241,7 @@
         <v>120</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E43" s="7" t="s">
         <v>6</v>
@@ -2267,7 +2258,7 @@
         <v>122</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>68</v>
+        <v>116</v>
       </c>
       <c r="E44" s="7" t="s">
         <v>6</v>
@@ -2284,7 +2275,7 @@
         <v>124</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>91</v>
+        <v>23</v>
       </c>
       <c r="E45" s="7" t="s">
         <v>6</v>
@@ -2301,7 +2292,7 @@
         <v>126</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>127</v>
+        <v>62</v>
       </c>
       <c r="E46" s="7" t="s">
         <v>6</v>
@@ -2309,16 +2300,16 @@
     </row>
     <row r="47" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="B47" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C47" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="B47" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C47" s="13" t="s">
-        <v>129</v>
-      </c>
       <c r="D47" s="13" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="E47" s="7" t="s">
         <v>6</v>
@@ -2326,16 +2317,16 @@
     </row>
     <row r="48" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="B48" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C48" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="B48" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C48" s="13" t="s">
-        <v>131</v>
-      </c>
       <c r="D48" s="13" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="E48" s="7" t="s">
         <v>6</v>
@@ -2343,16 +2334,16 @@
     </row>
     <row r="49" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="B49" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C49" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="B49" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C49" s="13" t="s">
-        <v>133</v>
-      </c>
       <c r="D49" s="13" t="s">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="E49" s="7" t="s">
         <v>6</v>
@@ -2360,16 +2351,16 @@
     </row>
     <row r="50" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="B50" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C50" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="B50" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C50" s="13" t="s">
-        <v>135</v>
-      </c>
       <c r="D50" s="13" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="E50" s="7" t="s">
         <v>6</v>
@@ -2377,16 +2368,16 @@
     </row>
     <row r="51" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="B51" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C51" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="B51" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C51" s="13" t="s">
-        <v>137</v>
-      </c>
       <c r="D51" s="13" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="E51" s="7" t="s">
         <v>6</v>
@@ -2394,16 +2385,16 @@
     </row>
     <row r="52" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="B52" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C52" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="B52" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C52" s="13" t="s">
-        <v>139</v>
-      </c>
       <c r="D52" s="13" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="E52" s="7" t="s">
         <v>6</v>
@@ -2411,13 +2402,13 @@
     </row>
     <row r="53" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="B53" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C53" s="13" t="s">
         <v>140</v>
-      </c>
-      <c r="B53" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C53" s="13" t="s">
-        <v>141</v>
       </c>
       <c r="D53" s="13" t="s">
         <v>38</v>
@@ -2428,16 +2419,16 @@
     </row>
     <row r="54" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="B54" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C54" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="B54" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C54" s="13" t="s">
-        <v>143</v>
-      </c>
       <c r="D54" s="13" t="s">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="E54" s="7" t="s">
         <v>6</v>
@@ -2445,16 +2436,16 @@
     </row>
     <row r="55" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="B55" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C55" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="B55" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C55" s="13" t="s">
-        <v>145</v>
-      </c>
       <c r="D55" s="13" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="E55" s="7" t="s">
         <v>6</v>
@@ -2462,16 +2453,16 @@
     </row>
     <row r="56" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="B56" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C56" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="B56" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C56" s="13" t="s">
-        <v>147</v>
-      </c>
       <c r="D56" s="13" t="s">
-        <v>103</v>
+        <v>72</v>
       </c>
       <c r="E56" s="7" t="s">
         <v>6</v>
@@ -2479,16 +2470,16 @@
     </row>
     <row r="57" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="B57" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C57" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="B57" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C57" s="13" t="s">
-        <v>149</v>
-      </c>
       <c r="D57" s="13" t="s">
-        <v>112</v>
+        <v>59</v>
       </c>
       <c r="E57" s="7" t="s">
         <v>6</v>
@@ -2496,16 +2487,16 @@
     </row>
     <row r="58" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="B58" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C58" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="B58" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C58" s="13" t="s">
-        <v>151</v>
-      </c>
       <c r="D58" s="13" t="s">
-        <v>35</v>
+        <v>94</v>
       </c>
       <c r="E58" s="7" t="s">
         <v>6</v>
@@ -2513,16 +2504,16 @@
     </row>
     <row r="59" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="B59" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C59" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="B59" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C59" s="13" t="s">
-        <v>153</v>
-      </c>
       <c r="D59" s="13" t="s">
-        <v>35</v>
+        <v>84</v>
       </c>
       <c r="E59" s="7" t="s">
         <v>6</v>
@@ -2530,16 +2521,16 @@
     </row>
     <row r="60" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="B60" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C60" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="B60" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C60" s="13" t="s">
-        <v>155</v>
-      </c>
       <c r="D60" s="13" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="E60" s="7" t="s">
         <v>6</v>
@@ -2547,16 +2538,16 @@
     </row>
     <row r="61" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="B61" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C61" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="B61" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C61" s="13" t="s">
-        <v>157</v>
-      </c>
       <c r="D61" s="13" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="E61" s="7" t="s">
         <v>6</v>
@@ -2564,16 +2555,16 @@
     </row>
     <row r="62" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="B62" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C62" s="13" t="s">
         <v>158</v>
       </c>
-      <c r="B62" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C62" s="13" t="s">
-        <v>159</v>
-      </c>
       <c r="D62" s="13" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="E62" s="7" t="s">
         <v>6</v>
@@ -2581,16 +2572,16 @@
     </row>
     <row r="63" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="B63" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C63" s="13" t="s">
         <v>160</v>
       </c>
-      <c r="B63" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C63" s="13" t="s">
-        <v>161</v>
-      </c>
       <c r="D63" s="13" t="s">
-        <v>162</v>
+        <v>26</v>
       </c>
       <c r="E63" s="7" t="s">
         <v>6</v>
@@ -2598,16 +2589,16 @@
     </row>
     <row r="64" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="B64" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C64" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="D64" s="13" t="s">
         <v>163</v>
-      </c>
-      <c r="B64" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C64" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="D64" s="13" t="s">
-        <v>100</v>
       </c>
       <c r="E64" s="7" t="s">
         <v>6</v>
@@ -2615,16 +2606,16 @@
     </row>
     <row r="65" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="13" t="s">
+        <v>164</v>
+      </c>
+      <c r="B65" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C65" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="B65" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C65" s="13" t="s">
-        <v>166</v>
-      </c>
       <c r="D65" s="13" t="s">
-        <v>26</v>
+        <v>94</v>
       </c>
       <c r="E65" s="7" t="s">
         <v>6</v>
@@ -2632,16 +2623,16 @@
     </row>
     <row r="66" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="B66" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C66" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="B66" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C66" s="13" t="s">
-        <v>168</v>
-      </c>
       <c r="D66" s="13" t="s">
-        <v>169</v>
+        <v>62</v>
       </c>
       <c r="E66" s="7" t="s">
         <v>6</v>
@@ -2649,16 +2640,16 @@
     </row>
     <row r="67" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="B67" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="C67" s="13" t="s">
         <v>170</v>
       </c>
-      <c r="B67" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="C67" s="13" t="s">
-        <v>172</v>
-      </c>
       <c r="D67" s="13" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="E67" s="7" t="s">
         <v>6</v>
@@ -2666,16 +2657,16 @@
     </row>
     <row r="68" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="13" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B68" s="13" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C68" s="13" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D68" s="13" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="E68" s="7" t="s">
         <v>6</v>
@@ -2683,16 +2674,16 @@
     </row>
     <row r="69" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="13" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B69" s="13" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C69" s="13" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D69" s="13" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="E69" s="7" t="s">
         <v>6</v>
@@ -2700,16 +2691,16 @@
     </row>
     <row r="70" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="B70" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="C70" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="D70" s="13" t="s">
         <v>178</v>
-      </c>
-      <c r="B70" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="C70" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="D70" s="13" t="s">
-        <v>112</v>
       </c>
       <c r="E70" s="7" t="s">
         <v>6</v>
@@ -2717,16 +2708,16 @@
     </row>
     <row r="71" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="B71" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="C71" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="B71" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="C71" s="13" t="s">
+      <c r="D71" s="13" t="s">
         <v>181</v>
-      </c>
-      <c r="D71" s="13" t="s">
-        <v>78</v>
       </c>
       <c r="E71" s="7" t="s">
         <v>6</v>
@@ -2737,13 +2728,13 @@
         <v>182</v>
       </c>
       <c r="B72" s="13" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C72" s="13" t="s">
         <v>183</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>51</v>
+        <v>163</v>
       </c>
       <c r="E72" s="7" t="s">
         <v>6</v>
@@ -2754,13 +2745,13 @@
         <v>184</v>
       </c>
       <c r="B73" s="13" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C73" s="13" t="s">
         <v>185</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>173</v>
+        <v>44</v>
       </c>
       <c r="E73" s="7" t="s">
         <v>6</v>
@@ -2771,7 +2762,7 @@
         <v>186</v>
       </c>
       <c r="B74" s="13" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C74" s="13" t="s">
         <v>187</v>
@@ -2788,13 +2779,13 @@
         <v>189</v>
       </c>
       <c r="B75" s="13" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C75" s="13" t="s">
         <v>190</v>
       </c>
       <c r="D75" s="13" t="s">
-        <v>191</v>
+        <v>89</v>
       </c>
       <c r="E75" s="7" t="s">
         <v>6</v>
@@ -2802,16 +2793,16 @@
     </row>
     <row r="76" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="B76" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="C76" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="B76" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="C76" s="13" t="s">
+      <c r="D76" s="13" t="s">
         <v>193</v>
-      </c>
-      <c r="D76" s="13" t="s">
-        <v>194</v>
       </c>
       <c r="E76" s="7" t="s">
         <v>6</v>
@@ -2819,16 +2810,16 @@
     </row>
     <row r="77" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="B77" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="B77" s="13" t="s">
+      <c r="C77" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="C77" s="13" t="s">
+      <c r="D77" s="13" t="s">
         <v>197</v>
-      </c>
-      <c r="D77" s="13" t="s">
-        <v>198</v>
       </c>
       <c r="E77" s="7" t="s">
         <v>6</v>
@@ -2836,16 +2827,16 @@
     </row>
     <row r="78" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="B78" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="B78" s="13" t="s">
+      <c r="C78" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="C78" s="13" t="s">
-        <v>201</v>
-      </c>
       <c r="D78" s="13" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="E78" s="7" t="s">
         <v>6</v>
@@ -2853,16 +2844,16 @@
     </row>
     <row r="79" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="B79" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="C79" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="B79" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="C79" s="13" t="s">
-        <v>203</v>
-      </c>
       <c r="D79" s="13" t="s">
-        <v>204</v>
+        <v>41</v>
       </c>
       <c r="E79" s="7" t="s">
         <v>6</v>
@@ -2870,16 +2861,16 @@
     </row>
     <row r="80" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="13" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B80" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="D80" s="13" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="E80" s="7" t="s">
         <v>6</v>
@@ -2887,16 +2878,16 @@
     </row>
     <row r="81" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="B81" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="C81" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="B81" s="13" t="s">
-        <v>208</v>
-      </c>
-      <c r="C81" s="13" t="s">
-        <v>209</v>
-      </c>
       <c r="D81" s="13" t="s">
-        <v>68</v>
+        <v>89</v>
       </c>
       <c r="E81" s="7" t="s">
         <v>6</v>
@@ -2904,16 +2895,16 @@
     </row>
     <row r="82" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="13" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B82" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C82" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D82" s="13" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E82" s="7" t="s">
         <v>6</v>
@@ -2921,16 +2912,16 @@
     </row>
     <row r="83" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="B83" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="C83" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D83" s="13" t="s">
         <v>212</v>
-      </c>
-      <c r="B83" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="C83" s="13" t="s">
-        <v>213</v>
-      </c>
-      <c r="D83" s="13" t="s">
-        <v>23</v>
       </c>
       <c r="E83" s="7" t="s">
         <v>6</v>
@@ -2938,16 +2929,16 @@
     </row>
     <row r="84" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="B84" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="C84" s="13" t="s">
         <v>214</v>
       </c>
-      <c r="B84" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="C84" s="13" t="s">
-        <v>215</v>
-      </c>
       <c r="D84" s="13" t="s">
-        <v>216</v>
+        <v>72</v>
       </c>
       <c r="E84" s="7" t="s">
         <v>6</v>
@@ -2955,16 +2946,16 @@
     </row>
     <row r="85" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="13" t="s">
+        <v>215</v>
+      </c>
+      <c r="B85" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="C85" s="13" t="s">
+        <v>216</v>
+      </c>
+      <c r="D85" s="13" t="s">
         <v>217</v>
-      </c>
-      <c r="B85" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="C85" s="13" t="s">
-        <v>218</v>
-      </c>
-      <c r="D85" s="13" t="s">
-        <v>68</v>
       </c>
       <c r="E85" s="7" t="s">
         <v>6</v>
@@ -2972,16 +2963,16 @@
     </row>
     <row r="86" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="B86" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="C86" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="B86" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="C86" s="13" t="s">
-        <v>220</v>
-      </c>
       <c r="D86" s="13" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="E86" s="7" t="s">
         <v>6</v>
@@ -2989,16 +2980,16 @@
     </row>
     <row r="87" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="13" t="s">
+        <v>220</v>
+      </c>
+      <c r="B87" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="C87" s="13" t="s">
         <v>221</v>
       </c>
-      <c r="B87" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="C87" s="13" t="s">
-        <v>222</v>
-      </c>
       <c r="D87" s="13" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="E87" s="7" t="s">
         <v>6</v>
@@ -3006,16 +2997,16 @@
     </row>
     <row r="88" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="13" t="s">
+        <v>222</v>
+      </c>
+      <c r="B88" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="C88" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="B88" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="C88" s="13" t="s">
-        <v>224</v>
-      </c>
       <c r="D88" s="13" t="s">
-        <v>216</v>
+        <v>116</v>
       </c>
       <c r="E88" s="7" t="s">
         <v>6</v>
@@ -3023,16 +3014,16 @@
     </row>
     <row r="89" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="13" t="s">
+        <v>224</v>
+      </c>
+      <c r="B89" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="C89" s="13" t="s">
         <v>225</v>
       </c>
-      <c r="B89" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="C89" s="13" t="s">
-        <v>226</v>
-      </c>
       <c r="D89" s="13" t="s">
-        <v>68</v>
+        <v>217</v>
       </c>
       <c r="E89" s="7" t="s">
         <v>6</v>
@@ -3040,16 +3031,16 @@
     </row>
     <row r="90" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="B90" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="C90" s="13" t="s">
         <v>227</v>
       </c>
-      <c r="B90" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="C90" s="13" t="s">
-        <v>228</v>
-      </c>
       <c r="D90" s="13" t="s">
-        <v>91</v>
+        <v>217</v>
       </c>
       <c r="E90" s="7" t="s">
         <v>6</v>
@@ -3057,16 +3048,16 @@
     </row>
     <row r="91" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="B91" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="C91" s="13" t="s">
         <v>229</v>
       </c>
-      <c r="B91" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="C91" s="13" t="s">
-        <v>230</v>
-      </c>
       <c r="D91" s="13" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="E91" s="7" t="s">
         <v>6</v>
@@ -3074,16 +3065,16 @@
     </row>
     <row r="92" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="13" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B92" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C92" s="13" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D92" s="13" t="s">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="E92" s="7" t="s">
         <v>6</v>
@@ -3091,16 +3082,16 @@
     </row>
     <row r="93" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="13" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B93" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C93" s="13" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="D93" s="13" t="s">
-        <v>236</v>
+        <v>72</v>
       </c>
       <c r="E93" s="7" t="s">
         <v>6</v>
@@ -3108,16 +3099,16 @@
     </row>
     <row r="94" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="13" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B94" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C94" s="13" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D94" s="13" t="s">
-        <v>38</v>
+        <v>89</v>
       </c>
       <c r="E94" s="7" t="s">
         <v>6</v>
@@ -3125,16 +3116,16 @@
     </row>
     <row r="95" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="13" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="B95" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C95" s="13" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D95" s="13" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="E95" s="7" t="s">
         <v>6</v>
@@ -3142,16 +3133,16 @@
     </row>
     <row r="96" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="13" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B96" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C96" s="13" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D96" s="13" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="E96" s="7" t="s">
         <v>6</v>
@@ -3159,16 +3150,16 @@
     </row>
     <row r="97" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="13" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="B97" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C97" s="13" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="D97" s="13" t="s">
-        <v>100</v>
+        <v>163</v>
       </c>
       <c r="E97" s="7" t="s">
         <v>6</v>
@@ -3176,16 +3167,16 @@
     </row>
     <row r="98" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="13" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B98" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C98" s="13" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D98" s="13" t="s">
-        <v>216</v>
+        <v>75</v>
       </c>
       <c r="E98" s="7" t="s">
         <v>6</v>
@@ -3193,16 +3184,16 @@
     </row>
     <row r="99" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="13" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B99" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C99" s="13" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D99" s="13" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E99" s="7" t="s">
         <v>6</v>
@@ -3210,16 +3201,16 @@
     </row>
     <row r="100" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="13" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="B100" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C100" s="13" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D100" s="13" t="s">
-        <v>75</v>
+        <v>41</v>
       </c>
       <c r="E100" s="7" t="s">
         <v>6</v>
@@ -3227,16 +3218,16 @@
     </row>
     <row r="101" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="13" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="B101" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C101" s="13" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D101" s="13" t="s">
-        <v>103</v>
+        <v>163</v>
       </c>
       <c r="E101" s="7" t="s">
         <v>6</v>
@@ -3244,16 +3235,16 @@
     </row>
     <row r="102" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="13" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B102" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C102" s="13" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D102" s="13" t="s">
-        <v>103</v>
+        <v>212</v>
       </c>
       <c r="E102" s="7" t="s">
         <v>6</v>
@@ -3261,16 +3252,16 @@
     </row>
     <row r="103" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="13" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B103" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C103" s="13" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="D103" s="13" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="E103" s="7" t="s">
         <v>6</v>
@@ -3278,16 +3269,16 @@
     </row>
     <row r="104" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="13" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="B104" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C104" s="13" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D104" s="13" t="s">
-        <v>100</v>
+        <v>163</v>
       </c>
       <c r="E104" s="7" t="s">
         <v>6</v>
@@ -3295,16 +3286,16 @@
     </row>
     <row r="105" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="13" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B105" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C105" s="13" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="D105" s="13" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="E105" s="7" t="s">
         <v>6</v>
@@ -3312,16 +3303,16 @@
     </row>
     <row r="106" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="13" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="B106" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C106" s="13" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D106" s="13" t="s">
-        <v>46</v>
+        <v>116</v>
       </c>
       <c r="E106" s="7" t="s">
         <v>6</v>
@@ -3329,16 +3320,16 @@
     </row>
     <row r="107" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="13" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="B107" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C107" s="13" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D107" s="13" t="s">
-        <v>38</v>
+        <v>65</v>
       </c>
       <c r="E107" s="7" t="s">
         <v>6</v>
@@ -3346,16 +3337,16 @@
     </row>
     <row r="108" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="13" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B108" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C108" s="13" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="D108" s="13" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="E108" s="7" t="s">
         <v>6</v>
@@ -3363,16 +3354,16 @@
     </row>
     <row r="109" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="13" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B109" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C109" s="13" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="D109" s="13" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="E109" s="7" t="s">
         <v>6</v>
@@ -3380,16 +3371,16 @@
     </row>
     <row r="110" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="13" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="B110" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C110" s="13" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D110" s="13" t="s">
-        <v>127</v>
+        <v>78</v>
       </c>
       <c r="E110" s="7" t="s">
         <v>6</v>
@@ -3397,16 +3388,16 @@
     </row>
     <row r="111" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="13" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B111" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C111" s="13" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D111" s="13" t="s">
-        <v>169</v>
+        <v>89</v>
       </c>
       <c r="E111" s="7" t="s">
         <v>6</v>
@@ -3414,16 +3405,16 @@
     </row>
     <row r="112" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="13" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="B112" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C112" s="13" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="D112" s="13" t="s">
-        <v>29</v>
+        <v>212</v>
       </c>
       <c r="E112" s="7" t="s">
         <v>6</v>
@@ -3431,16 +3422,16 @@
     </row>
     <row r="113" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="13" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="B113" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C113" s="13" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="D113" s="13" t="s">
-        <v>269</v>
+        <v>38</v>
       </c>
       <c r="E113" s="7" t="s">
         <v>6</v>
@@ -3448,16 +3439,16 @@
     </row>
     <row r="114" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="13" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B114" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C114" s="13" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D114" s="13" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="E114" s="7" t="s">
         <v>6</v>
@@ -3465,16 +3456,16 @@
     </row>
     <row r="115" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="13" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B115" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C115" s="13" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="D115" s="13" t="s">
-        <v>32</v>
+        <v>163</v>
       </c>
       <c r="E115" s="7" t="s">
         <v>6</v>
@@ -3482,16 +3473,16 @@
     </row>
     <row r="116" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="13" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="B116" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C116" s="13" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="D116" s="13" t="s">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="E116" s="7" t="s">
         <v>6</v>
@@ -3499,16 +3490,16 @@
     </row>
     <row r="117" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="13" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="B117" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C117" s="13" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="D117" s="13" t="s">
-        <v>286</v>
+        <v>163</v>
       </c>
       <c r="E117" s="7" t="s">
         <v>6</v>
@@ -3516,16 +3507,16 @@
     </row>
     <row r="118" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="13" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="B118" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C118" s="13" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="D118" s="13" t="s">
-        <v>169</v>
+        <v>89</v>
       </c>
       <c r="E118" s="7" t="s">
         <v>6</v>
@@ -3533,16 +3524,16 @@
     </row>
     <row r="119" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="13" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B119" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C119" s="13" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="D119" s="13" t="s">
-        <v>118</v>
+        <v>44</v>
       </c>
       <c r="E119" s="7" t="s">
         <v>6</v>
@@ -3550,13 +3541,13 @@
     </row>
     <row r="120" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="13" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="B120" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C120" s="13" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="D120" s="13" t="s">
         <v>26</v>
@@ -3567,16 +3558,16 @@
     </row>
     <row r="121" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="13" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="B121" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C121" s="13" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="D121" s="13" t="s">
-        <v>169</v>
+        <v>291</v>
       </c>
       <c r="E121" s="7" t="s">
         <v>6</v>
@@ -3584,16 +3575,16 @@
     </row>
     <row r="122" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="13" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="B122" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C122" s="13" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D122" s="13" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="E122" s="7" t="s">
         <v>6</v>
@@ -3601,16 +3592,16 @@
     </row>
     <row r="123" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="13" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B123" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C123" s="13" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D123" s="13" t="s">
-        <v>118</v>
+        <v>81</v>
       </c>
       <c r="E123" s="7" t="s">
         <v>6</v>
@@ -3618,16 +3609,16 @@
     </row>
     <row r="124" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="13" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="B124" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C124" s="13" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="D124" s="13" t="s">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="E124" s="7" t="s">
         <v>6</v>
@@ -3635,16 +3626,16 @@
     </row>
     <row r="125" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="13" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="B125" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C125" s="13" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="D125" s="13" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="E125" s="7" t="s">
         <v>6</v>
@@ -3652,16 +3643,16 @@
     </row>
     <row r="126" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="13" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="B126" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C126" s="13" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="D126" s="13" t="s">
-        <v>100</v>
+        <v>23</v>
       </c>
       <c r="E126" s="7" t="s">
         <v>6</v>
@@ -3669,16 +3660,16 @@
     </row>
     <row r="127" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="13" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="B127" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C127" s="13" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="D127" s="13" t="s">
-        <v>127</v>
+        <v>89</v>
       </c>
       <c r="E127" s="7" t="s">
         <v>6</v>
@@ -3686,16 +3677,16 @@
     </row>
     <row r="128" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="13" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="B128" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C128" s="13" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="D128" s="13" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="E128" s="7" t="s">
         <v>6</v>

</xml_diff>